<commit_message>
Addes Manually Observation regarding the Dataset
</commit_message>
<xml_diff>
--- a/output.xlsx
+++ b/output.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RonitJadhav\Personal\01_Learning\Python\Code\Pandas\Projects\Pandas_GitHub\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44E5AFCA-CA89-4CA4-B1B7-A99E88A664A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{805E487F-F1DF-486F-9C74-01728ED1D055}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="patients" sheetId="1" r:id="rId1"/>
@@ -33635,6 +33635,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:G281"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="17.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="8.54296875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.7265625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">

</xml_diff>